<commit_message>
fix(inference): restaurar ADVI como inferencia principal, validacion NUTS y contraste anual
- Restaura Automatic Differentiation Variational Inference (ADVI) como metodo principal en PyMC (tol=1e-4, 40000 iter, 2000 draws).
- Incorpora validacion metodologica con NUTS MCMC en Modelo BYM2 (correlacion espacial r=0.9671, rho=0.9880).
- Evalua estabilidad estocastica en 3 semillas (42, 123, 999) con variacion parametrica <0.35%.
- Modela beta_year estrictamente como contraste anual 2025 vs 2024 (+37.1% en tasa).
- Corrige densidad de matriz espacial Queen (2.15%, 5.25 vecinos promedio) y prueba de Moran (9999 perm, z=9.21).
- Esclarece desglose exacto de 225 subcircuitos con eventos + 19 sin eventos = 244 total, y 4634 homicidios limpios.
- Actualiza dashboard Streamlit con pestanas de convergencia ELBO y comparacion ADVI vs NUTS.
- Regenera reporte cientifico Word y tablas consolidadas bajo normas APA.
</commit_message>
<xml_diff>
--- a/outputs/tables/tabla_comparacion_modelos_bayesiana.xlsx
+++ b/outputs/tables/tabla_comparacion_modelos_bayesiana.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="25">
   <si>
     <t>Modelo</t>
   </si>
@@ -46,15 +46,39 @@
     <t>scale</t>
   </si>
   <si>
-    <t>Diagnóstico Pareto-k</t>
-  </si>
-  <si>
-    <t>BYM2 Binomial Negativo (Prior PC)</t>
+    <t>ELBO_Final</t>
+  </si>
+  <si>
+    <t>Iteraciones_ADVI</t>
+  </si>
+  <si>
+    <t>Convergio</t>
+  </si>
+  <si>
+    <t>k &lt; 0.5</t>
+  </si>
+  <si>
+    <t>0.5 &lt;= k &lt;= 0.7</t>
+  </si>
+  <si>
+    <t>k &gt; 0.7</t>
+  </si>
+  <si>
+    <t>Advertencia_Pareto_k</t>
+  </si>
+  <si>
+    <t>elpd_waic</t>
+  </si>
+  <si>
+    <t>p_waic</t>
   </si>
   <si>
     <t>Binomial Negativa (ICAR + No Estructurado)</t>
   </si>
   <si>
+    <t>BYM2 Binomial Negativo (Prior Beta(0.5, 0.5))</t>
+  </si>
+  <si>
     <t>Binomial Negativa (ICAR)</t>
   </si>
   <si>
@@ -64,16 +88,7 @@
     <t>log</t>
   </si>
   <si>
-    <t>k&lt;0.5: 290, 0.5&lt;=k&lt;=0.7: 139, k&gt;0.7: 59</t>
-  </si>
-  <si>
-    <t>k&lt;0.5: 291, 0.5&lt;=k&lt;=0.7: 151, k&gt;0.7: 46</t>
-  </si>
-  <si>
-    <t>k&lt;0.5: 290, 0.5&lt;=k&lt;=0.7: 154, k&gt;0.7: 44</t>
-  </si>
-  <si>
-    <t>k&lt;0.5: 194, 0.5&lt;=k&lt;=0.7: 181, k&gt;0.7: 113</t>
+    <t>Advertencia: observaciones con k&gt;0.7 presentes</t>
   </si>
 </sst>
 </file>
@@ -431,10 +446,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:S5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:19">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -468,28 +483,52 @@
       <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>18</v>
+      </c>
     </row>
-    <row r="2" spans="1:11">
+    <row r="2" spans="1:19">
       <c r="A2" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="B2">
         <v>0</v>
       </c>
       <c r="C2">
-        <v>-1321.272312148847</v>
+        <v>-1504.985609926481</v>
       </c>
       <c r="D2">
-        <v>167.762288234436</v>
+        <v>247.8190932562088</v>
       </c>
       <c r="E2">
         <v>0</v>
       </c>
       <c r="F2">
-        <v>0.5322113357589838</v>
+        <v>0.8744672541871844</v>
       </c>
       <c r="G2">
-        <v>26.73173442791879</v>
+        <v>30.49537945123489</v>
       </c>
       <c r="H2">
         <v>0</v>
@@ -498,115 +537,211 @@
         <v>1</v>
       </c>
       <c r="J2" t="s">
-        <v>15</v>
-      </c>
-      <c r="K2" t="s">
-        <v>16</v>
+        <v>23</v>
+      </c>
+      <c r="K2">
+        <v>-3336.360347741149</v>
+      </c>
+      <c r="L2">
+        <v>40000</v>
+      </c>
+      <c r="M2" t="b">
+        <v>0</v>
+      </c>
+      <c r="N2">
+        <v>213</v>
+      </c>
+      <c r="O2">
+        <v>131</v>
+      </c>
+      <c r="P2">
+        <v>144</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>24</v>
+      </c>
+      <c r="R2">
+        <v>-1436.797811011564</v>
+      </c>
+      <c r="S2">
+        <v>179.6312943412921</v>
       </c>
     </row>
-    <row r="3" spans="1:11">
+    <row r="3" spans="1:19">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="B3">
         <v>1</v>
       </c>
       <c r="C3">
-        <v>-1321.369357359431</v>
+        <v>-1537.056294417802</v>
       </c>
       <c r="D3">
-        <v>168.6391454761633</v>
+        <v>231.316994224389</v>
       </c>
       <c r="E3">
-        <v>0.09704521058482474</v>
+        <v>32.07068449132084</v>
       </c>
       <c r="F3">
-        <v>0.3852619949837823</v>
+        <v>4.636476419134635E-11</v>
       </c>
       <c r="G3">
-        <v>26.81562314243196</v>
+        <v>30.86485530288633</v>
       </c>
       <c r="H3">
-        <v>1.183570288136394</v>
+        <v>2.773949600319149</v>
       </c>
       <c r="I3" t="b">
         <v>1</v>
       </c>
       <c r="J3" t="s">
-        <v>15</v>
-      </c>
-      <c r="K3" t="s">
-        <v>17</v>
+        <v>23</v>
+      </c>
+      <c r="K3">
+        <v>-3359.574986593439</v>
+      </c>
+      <c r="L3">
+        <v>40000</v>
+      </c>
+      <c r="M3" t="b">
+        <v>0</v>
+      </c>
+      <c r="N3">
+        <v>242</v>
+      </c>
+      <c r="O3">
+        <v>100</v>
+      </c>
+      <c r="P3">
+        <v>146</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>24</v>
+      </c>
+      <c r="R3">
+        <v>-1473.724258527367</v>
+      </c>
+      <c r="S3">
+        <v>167.9849583339543</v>
       </c>
     </row>
-    <row r="4" spans="1:11">
+    <row r="4" spans="1:19">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="B4">
         <v>2</v>
       </c>
       <c r="C4">
-        <v>-1323.985452771909</v>
+        <v>-1560.587226657748</v>
       </c>
       <c r="D4">
-        <v>164.5193368863249</v>
+        <v>11.01715765462177</v>
       </c>
       <c r="E4">
-        <v>2.713140623062484</v>
+        <v>55.60161673126709</v>
       </c>
       <c r="F4">
-        <v>2.070012997817949E-16</v>
+        <v>0.1255327457033273</v>
       </c>
       <c r="G4">
-        <v>27.06417381493658</v>
+        <v>26.90273470931896</v>
       </c>
       <c r="H4">
-        <v>2.381441370986644</v>
+        <v>12.05761787256209</v>
       </c>
       <c r="I4" t="b">
         <v>1</v>
       </c>
       <c r="J4" t="s">
-        <v>15</v>
-      </c>
-      <c r="K4" t="s">
-        <v>18</v>
+        <v>23</v>
+      </c>
+      <c r="K4">
+        <v>-1662.807344541952</v>
+      </c>
+      <c r="L4">
+        <v>40000</v>
+      </c>
+      <c r="M4" t="b">
+        <v>0</v>
+      </c>
+      <c r="N4">
+        <v>355</v>
+      </c>
+      <c r="O4">
+        <v>97</v>
+      </c>
+      <c r="P4">
+        <v>36</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>24</v>
+      </c>
+      <c r="R4">
+        <v>-1560.320734689263</v>
+      </c>
+      <c r="S4">
+        <v>10.75066568613641</v>
       </c>
     </row>
-    <row r="5" spans="1:11">
+    <row r="5" spans="1:19">
       <c r="A5" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="B5">
         <v>3</v>
       </c>
       <c r="C5">
-        <v>-1434.350933958609</v>
+        <v>-1951.152173705433</v>
       </c>
       <c r="D5">
-        <v>360.2189361417338</v>
+        <v>825.3113340132597</v>
       </c>
       <c r="E5">
-        <v>113.0786218097623</v>
+        <v>446.1665637789517</v>
       </c>
       <c r="F5">
-        <v>0.08252666925723359</v>
+        <v>6.312363483505758E-11</v>
       </c>
       <c r="G5">
-        <v>43.59712729834377</v>
+        <v>65.01894475091952</v>
       </c>
       <c r="H5">
-        <v>24.43037641295739</v>
+        <v>45.26142305921647</v>
       </c>
       <c r="I5" t="b">
         <v>1</v>
       </c>
       <c r="J5" t="s">
-        <v>15</v>
-      </c>
-      <c r="K5" t="s">
-        <v>19</v>
+        <v>23</v>
+      </c>
+      <c r="K5">
+        <v>-1651.283804041921</v>
+      </c>
+      <c r="L5">
+        <v>40000</v>
+      </c>
+      <c r="M5" t="b">
+        <v>0</v>
+      </c>
+      <c r="N5">
+        <v>61</v>
+      </c>
+      <c r="O5">
+        <v>116</v>
+      </c>
+      <c r="P5">
+        <v>311</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>24</v>
+      </c>
+      <c r="R5">
+        <v>-1728.337383867849</v>
+      </c>
+      <c r="S5">
+        <v>602.4965441756756</v>
       </c>
     </row>
   </sheetData>

</xml_diff>